<commit_message>
Create pydantic model for general input
</commit_message>
<xml_diff>
--- a/tests/fmudesign/data/config/design_input_onebyone.xlsx
+++ b/tests/fmudesign/data/config/design_input_onebyone.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="11110"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="10713"/>
   <workbookPr defaultThemeVersion="202300"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/FCUR/git/semeio/tests/fmudesign/data/config/"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/SKAV/git_repos/semeio/tests/fmudesign/data/config/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{CDC7CD35-9D11-9848-8278-0FE4092CA675}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{EDE762A3-5847-1248-B176-A8D2A43475C1}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="0" yWindow="500" windowWidth="32900" windowHeight="21620" tabRatio="500" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="0" yWindow="660" windowWidth="30240" windowHeight="18980" tabRatio="500" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="general_input" sheetId="1" r:id="rId1"/>
@@ -20,7 +20,7 @@
     <sheet name="background" sheetId="5" r:id="rId5"/>
     <sheet name="background_corr" sheetId="6" r:id="rId6"/>
   </sheets>
-  <calcPr calcId="0"/>
+  <calcPr calcId="0" iterateDelta="1E-4"/>
   <extLst>
     <ext xmlns:loext="http://schemas.libreoffice.org/" uri="{7626C862-2A13-11E5-B345-FEFF819CDC9F}">
       <loext:extCalcPr stringRefSyntax="CalcA1ExcelA1"/>
@@ -2134,6 +2134,222 @@
     </xdr:sp>
     <xdr:clientData/>
   </xdr:twoCellAnchor>
+  <xdr:twoCellAnchor>
+    <xdr:from>
+      <xdr:col>0</xdr:col>
+      <xdr:colOff>0</xdr:colOff>
+      <xdr:row>0</xdr:row>
+      <xdr:rowOff>0</xdr:rowOff>
+    </xdr:from>
+    <xdr:to>
+      <xdr:col>10</xdr:col>
+      <xdr:colOff>558800</xdr:colOff>
+      <xdr:row>66</xdr:row>
+      <xdr:rowOff>127000</xdr:rowOff>
+    </xdr:to>
+    <xdr:sp macro="" textlink="">
+      <xdr:nvSpPr>
+        <xdr:cNvPr id="2" name="AutoShape 8">
+          <a:extLst>
+            <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
+              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{E61F62A1-C8D0-1930-4470-661E75BF55FF}"/>
+            </a:ext>
+          </a:extLst>
+        </xdr:cNvPr>
+        <xdr:cNvSpPr>
+          <a:spLocks noChangeArrowheads="1"/>
+        </xdr:cNvSpPr>
+      </xdr:nvSpPr>
+      <xdr:spPr bwMode="auto">
+        <a:xfrm>
+          <a:off x="0" y="0"/>
+          <a:ext cx="13004800" cy="12700000"/>
+        </a:xfrm>
+        <a:custGeom>
+          <a:avLst/>
+          <a:gdLst/>
+          <a:ahLst/>
+          <a:cxnLst/>
+          <a:rect l="0" t="0" r="0" b="0"/>
+          <a:pathLst/>
+        </a:custGeom>
+        <a:solidFill>
+          <a:srgbClr val="FFFFFF"/>
+        </a:solidFill>
+        <a:ln w="9525">
+          <a:solidFill>
+            <a:srgbClr val="000000"/>
+          </a:solidFill>
+          <a:round/>
+          <a:headEnd/>
+          <a:tailEnd/>
+        </a:ln>
+      </xdr:spPr>
+    </xdr:sp>
+    <xdr:clientData/>
+  </xdr:twoCellAnchor>
+  <xdr:twoCellAnchor>
+    <xdr:from>
+      <xdr:col>0</xdr:col>
+      <xdr:colOff>0</xdr:colOff>
+      <xdr:row>0</xdr:row>
+      <xdr:rowOff>0</xdr:rowOff>
+    </xdr:from>
+    <xdr:to>
+      <xdr:col>10</xdr:col>
+      <xdr:colOff>558800</xdr:colOff>
+      <xdr:row>66</xdr:row>
+      <xdr:rowOff>127000</xdr:rowOff>
+    </xdr:to>
+    <xdr:sp macro="" textlink="">
+      <xdr:nvSpPr>
+        <xdr:cNvPr id="3" name="AutoShape 6">
+          <a:extLst>
+            <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
+              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{FFB291F9-2868-44AB-53CC-70FDF0EA437B}"/>
+            </a:ext>
+          </a:extLst>
+        </xdr:cNvPr>
+        <xdr:cNvSpPr>
+          <a:spLocks noChangeArrowheads="1"/>
+        </xdr:cNvSpPr>
+      </xdr:nvSpPr>
+      <xdr:spPr bwMode="auto">
+        <a:xfrm>
+          <a:off x="0" y="0"/>
+          <a:ext cx="13004800" cy="12700000"/>
+        </a:xfrm>
+        <a:custGeom>
+          <a:avLst/>
+          <a:gdLst/>
+          <a:ahLst/>
+          <a:cxnLst/>
+          <a:rect l="0" t="0" r="0" b="0"/>
+          <a:pathLst/>
+        </a:custGeom>
+        <a:solidFill>
+          <a:srgbClr val="FFFFFF"/>
+        </a:solidFill>
+        <a:ln w="9525">
+          <a:solidFill>
+            <a:srgbClr val="000000"/>
+          </a:solidFill>
+          <a:round/>
+          <a:headEnd/>
+          <a:tailEnd/>
+        </a:ln>
+      </xdr:spPr>
+    </xdr:sp>
+    <xdr:clientData/>
+  </xdr:twoCellAnchor>
+  <xdr:twoCellAnchor>
+    <xdr:from>
+      <xdr:col>0</xdr:col>
+      <xdr:colOff>0</xdr:colOff>
+      <xdr:row>0</xdr:row>
+      <xdr:rowOff>0</xdr:rowOff>
+    </xdr:from>
+    <xdr:to>
+      <xdr:col>10</xdr:col>
+      <xdr:colOff>558800</xdr:colOff>
+      <xdr:row>66</xdr:row>
+      <xdr:rowOff>127000</xdr:rowOff>
+    </xdr:to>
+    <xdr:sp macro="" textlink="">
+      <xdr:nvSpPr>
+        <xdr:cNvPr id="4" name="AutoShape 4">
+          <a:extLst>
+            <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
+              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{1689D2B9-D981-EB5D-8BAA-624F2E30D00F}"/>
+            </a:ext>
+          </a:extLst>
+        </xdr:cNvPr>
+        <xdr:cNvSpPr>
+          <a:spLocks noChangeArrowheads="1"/>
+        </xdr:cNvSpPr>
+      </xdr:nvSpPr>
+      <xdr:spPr bwMode="auto">
+        <a:xfrm>
+          <a:off x="0" y="0"/>
+          <a:ext cx="13004800" cy="12700000"/>
+        </a:xfrm>
+        <a:custGeom>
+          <a:avLst/>
+          <a:gdLst/>
+          <a:ahLst/>
+          <a:cxnLst/>
+          <a:rect l="0" t="0" r="0" b="0"/>
+          <a:pathLst/>
+        </a:custGeom>
+        <a:solidFill>
+          <a:srgbClr val="FFFFFF"/>
+        </a:solidFill>
+        <a:ln w="9525">
+          <a:solidFill>
+            <a:srgbClr val="000000"/>
+          </a:solidFill>
+          <a:round/>
+          <a:headEnd/>
+          <a:tailEnd/>
+        </a:ln>
+      </xdr:spPr>
+    </xdr:sp>
+    <xdr:clientData/>
+  </xdr:twoCellAnchor>
+  <xdr:twoCellAnchor>
+    <xdr:from>
+      <xdr:col>0</xdr:col>
+      <xdr:colOff>0</xdr:colOff>
+      <xdr:row>0</xdr:row>
+      <xdr:rowOff>0</xdr:rowOff>
+    </xdr:from>
+    <xdr:to>
+      <xdr:col>10</xdr:col>
+      <xdr:colOff>558800</xdr:colOff>
+      <xdr:row>66</xdr:row>
+      <xdr:rowOff>127000</xdr:rowOff>
+    </xdr:to>
+    <xdr:sp macro="" textlink="">
+      <xdr:nvSpPr>
+        <xdr:cNvPr id="5" name="AutoShape 2">
+          <a:extLst>
+            <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
+              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{E57A792A-D04E-A413-76CC-6587D7F8FCCD}"/>
+            </a:ext>
+          </a:extLst>
+        </xdr:cNvPr>
+        <xdr:cNvSpPr>
+          <a:spLocks noChangeArrowheads="1"/>
+        </xdr:cNvSpPr>
+      </xdr:nvSpPr>
+      <xdr:spPr bwMode="auto">
+        <a:xfrm>
+          <a:off x="0" y="0"/>
+          <a:ext cx="13004800" cy="12700000"/>
+        </a:xfrm>
+        <a:custGeom>
+          <a:avLst/>
+          <a:gdLst/>
+          <a:ahLst/>
+          <a:cxnLst/>
+          <a:rect l="0" t="0" r="0" b="0"/>
+          <a:pathLst/>
+        </a:custGeom>
+        <a:solidFill>
+          <a:srgbClr val="FFFFFF"/>
+        </a:solidFill>
+        <a:ln w="9525">
+          <a:solidFill>
+            <a:srgbClr val="000000"/>
+          </a:solidFill>
+          <a:round/>
+          <a:headEnd/>
+          <a:tailEnd/>
+        </a:ln>
+      </xdr:spPr>
+    </xdr:sp>
+    <xdr:clientData/>
+  </xdr:twoCellAnchor>
 </xdr:wsDr>
 </file>
 
@@ -2384,6 +2600,276 @@
     </xdr:sp>
     <xdr:clientData/>
   </xdr:twoCellAnchor>
+  <xdr:twoCellAnchor>
+    <xdr:from>
+      <xdr:col>0</xdr:col>
+      <xdr:colOff>0</xdr:colOff>
+      <xdr:row>0</xdr:row>
+      <xdr:rowOff>0</xdr:rowOff>
+    </xdr:from>
+    <xdr:to>
+      <xdr:col>12</xdr:col>
+      <xdr:colOff>558800</xdr:colOff>
+      <xdr:row>66</xdr:row>
+      <xdr:rowOff>127000</xdr:rowOff>
+    </xdr:to>
+    <xdr:sp macro="" textlink="">
+      <xdr:nvSpPr>
+        <xdr:cNvPr id="2" name="AutoShape 10">
+          <a:extLst>
+            <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
+              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{A3C7EB79-517A-CC44-4674-7392D1FB771E}"/>
+            </a:ext>
+          </a:extLst>
+        </xdr:cNvPr>
+        <xdr:cNvSpPr>
+          <a:spLocks noChangeArrowheads="1"/>
+        </xdr:cNvSpPr>
+      </xdr:nvSpPr>
+      <xdr:spPr bwMode="auto">
+        <a:xfrm>
+          <a:off x="0" y="0"/>
+          <a:ext cx="12700000" cy="12700000"/>
+        </a:xfrm>
+        <a:custGeom>
+          <a:avLst/>
+          <a:gdLst/>
+          <a:ahLst/>
+          <a:cxnLst/>
+          <a:rect l="0" t="0" r="0" b="0"/>
+          <a:pathLst/>
+        </a:custGeom>
+        <a:solidFill>
+          <a:srgbClr val="FFFFFF"/>
+        </a:solidFill>
+        <a:ln w="9525">
+          <a:solidFill>
+            <a:srgbClr val="000000"/>
+          </a:solidFill>
+          <a:round/>
+          <a:headEnd/>
+          <a:tailEnd/>
+        </a:ln>
+      </xdr:spPr>
+    </xdr:sp>
+    <xdr:clientData/>
+  </xdr:twoCellAnchor>
+  <xdr:twoCellAnchor>
+    <xdr:from>
+      <xdr:col>0</xdr:col>
+      <xdr:colOff>0</xdr:colOff>
+      <xdr:row>0</xdr:row>
+      <xdr:rowOff>0</xdr:rowOff>
+    </xdr:from>
+    <xdr:to>
+      <xdr:col>12</xdr:col>
+      <xdr:colOff>558800</xdr:colOff>
+      <xdr:row>66</xdr:row>
+      <xdr:rowOff>127000</xdr:rowOff>
+    </xdr:to>
+    <xdr:sp macro="" textlink="">
+      <xdr:nvSpPr>
+        <xdr:cNvPr id="3" name="AutoShape 8">
+          <a:extLst>
+            <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
+              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{F22A8815-1063-CDDD-67D4-F9906C48178F}"/>
+            </a:ext>
+          </a:extLst>
+        </xdr:cNvPr>
+        <xdr:cNvSpPr>
+          <a:spLocks noChangeArrowheads="1"/>
+        </xdr:cNvSpPr>
+      </xdr:nvSpPr>
+      <xdr:spPr bwMode="auto">
+        <a:xfrm>
+          <a:off x="0" y="0"/>
+          <a:ext cx="12700000" cy="12700000"/>
+        </a:xfrm>
+        <a:custGeom>
+          <a:avLst/>
+          <a:gdLst/>
+          <a:ahLst/>
+          <a:cxnLst/>
+          <a:rect l="0" t="0" r="0" b="0"/>
+          <a:pathLst/>
+        </a:custGeom>
+        <a:solidFill>
+          <a:srgbClr val="FFFFFF"/>
+        </a:solidFill>
+        <a:ln w="9525">
+          <a:solidFill>
+            <a:srgbClr val="000000"/>
+          </a:solidFill>
+          <a:round/>
+          <a:headEnd/>
+          <a:tailEnd/>
+        </a:ln>
+      </xdr:spPr>
+    </xdr:sp>
+    <xdr:clientData/>
+  </xdr:twoCellAnchor>
+  <xdr:twoCellAnchor>
+    <xdr:from>
+      <xdr:col>0</xdr:col>
+      <xdr:colOff>0</xdr:colOff>
+      <xdr:row>0</xdr:row>
+      <xdr:rowOff>0</xdr:rowOff>
+    </xdr:from>
+    <xdr:to>
+      <xdr:col>12</xdr:col>
+      <xdr:colOff>558800</xdr:colOff>
+      <xdr:row>66</xdr:row>
+      <xdr:rowOff>127000</xdr:rowOff>
+    </xdr:to>
+    <xdr:sp macro="" textlink="">
+      <xdr:nvSpPr>
+        <xdr:cNvPr id="4" name="AutoShape 6">
+          <a:extLst>
+            <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
+              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{DD534B41-C3EF-B28C-1E32-5FA831D6E36C}"/>
+            </a:ext>
+          </a:extLst>
+        </xdr:cNvPr>
+        <xdr:cNvSpPr>
+          <a:spLocks noChangeArrowheads="1"/>
+        </xdr:cNvSpPr>
+      </xdr:nvSpPr>
+      <xdr:spPr bwMode="auto">
+        <a:xfrm>
+          <a:off x="0" y="0"/>
+          <a:ext cx="12700000" cy="12700000"/>
+        </a:xfrm>
+        <a:custGeom>
+          <a:avLst/>
+          <a:gdLst/>
+          <a:ahLst/>
+          <a:cxnLst/>
+          <a:rect l="0" t="0" r="0" b="0"/>
+          <a:pathLst/>
+        </a:custGeom>
+        <a:solidFill>
+          <a:srgbClr val="FFFFFF"/>
+        </a:solidFill>
+        <a:ln w="9525">
+          <a:solidFill>
+            <a:srgbClr val="000000"/>
+          </a:solidFill>
+          <a:round/>
+          <a:headEnd/>
+          <a:tailEnd/>
+        </a:ln>
+      </xdr:spPr>
+    </xdr:sp>
+    <xdr:clientData/>
+  </xdr:twoCellAnchor>
+  <xdr:twoCellAnchor>
+    <xdr:from>
+      <xdr:col>0</xdr:col>
+      <xdr:colOff>0</xdr:colOff>
+      <xdr:row>0</xdr:row>
+      <xdr:rowOff>0</xdr:rowOff>
+    </xdr:from>
+    <xdr:to>
+      <xdr:col>12</xdr:col>
+      <xdr:colOff>558800</xdr:colOff>
+      <xdr:row>66</xdr:row>
+      <xdr:rowOff>127000</xdr:rowOff>
+    </xdr:to>
+    <xdr:sp macro="" textlink="">
+      <xdr:nvSpPr>
+        <xdr:cNvPr id="5" name="AutoShape 4">
+          <a:extLst>
+            <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
+              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{1A35FFE2-F966-9D8F-AE03-18589ADA3675}"/>
+            </a:ext>
+          </a:extLst>
+        </xdr:cNvPr>
+        <xdr:cNvSpPr>
+          <a:spLocks noChangeArrowheads="1"/>
+        </xdr:cNvSpPr>
+      </xdr:nvSpPr>
+      <xdr:spPr bwMode="auto">
+        <a:xfrm>
+          <a:off x="0" y="0"/>
+          <a:ext cx="12700000" cy="12700000"/>
+        </a:xfrm>
+        <a:custGeom>
+          <a:avLst/>
+          <a:gdLst/>
+          <a:ahLst/>
+          <a:cxnLst/>
+          <a:rect l="0" t="0" r="0" b="0"/>
+          <a:pathLst/>
+        </a:custGeom>
+        <a:solidFill>
+          <a:srgbClr val="FFFFFF"/>
+        </a:solidFill>
+        <a:ln w="9525">
+          <a:solidFill>
+            <a:srgbClr val="000000"/>
+          </a:solidFill>
+          <a:round/>
+          <a:headEnd/>
+          <a:tailEnd/>
+        </a:ln>
+      </xdr:spPr>
+    </xdr:sp>
+    <xdr:clientData/>
+  </xdr:twoCellAnchor>
+  <xdr:twoCellAnchor>
+    <xdr:from>
+      <xdr:col>0</xdr:col>
+      <xdr:colOff>0</xdr:colOff>
+      <xdr:row>0</xdr:row>
+      <xdr:rowOff>0</xdr:rowOff>
+    </xdr:from>
+    <xdr:to>
+      <xdr:col>12</xdr:col>
+      <xdr:colOff>558800</xdr:colOff>
+      <xdr:row>66</xdr:row>
+      <xdr:rowOff>127000</xdr:rowOff>
+    </xdr:to>
+    <xdr:sp macro="" textlink="">
+      <xdr:nvSpPr>
+        <xdr:cNvPr id="6" name="AutoShape 2">
+          <a:extLst>
+            <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
+              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{467B1236-5B88-B757-FF30-FE9D03D05E75}"/>
+            </a:ext>
+          </a:extLst>
+        </xdr:cNvPr>
+        <xdr:cNvSpPr>
+          <a:spLocks noChangeArrowheads="1"/>
+        </xdr:cNvSpPr>
+      </xdr:nvSpPr>
+      <xdr:spPr bwMode="auto">
+        <a:xfrm>
+          <a:off x="0" y="0"/>
+          <a:ext cx="12700000" cy="12700000"/>
+        </a:xfrm>
+        <a:custGeom>
+          <a:avLst/>
+          <a:gdLst/>
+          <a:ahLst/>
+          <a:cxnLst/>
+          <a:rect l="0" t="0" r="0" b="0"/>
+          <a:pathLst/>
+        </a:custGeom>
+        <a:solidFill>
+          <a:srgbClr val="FFFFFF"/>
+        </a:solidFill>
+        <a:ln w="9525">
+          <a:solidFill>
+            <a:srgbClr val="000000"/>
+          </a:solidFill>
+          <a:round/>
+          <a:headEnd/>
+          <a:tailEnd/>
+        </a:ln>
+      </xdr:spPr>
+    </xdr:sp>
+    <xdr:clientData/>
+  </xdr:twoCellAnchor>
 </xdr:wsDr>
 </file>
 
@@ -2438,6 +2924,60 @@
     </xdr:sp>
     <xdr:clientData/>
   </xdr:twoCellAnchor>
+  <xdr:twoCellAnchor>
+    <xdr:from>
+      <xdr:col>0</xdr:col>
+      <xdr:colOff>0</xdr:colOff>
+      <xdr:row>0</xdr:row>
+      <xdr:rowOff>0</xdr:rowOff>
+    </xdr:from>
+    <xdr:to>
+      <xdr:col>18</xdr:col>
+      <xdr:colOff>152400</xdr:colOff>
+      <xdr:row>66</xdr:row>
+      <xdr:rowOff>127000</xdr:rowOff>
+    </xdr:to>
+    <xdr:sp macro="" textlink="">
+      <xdr:nvSpPr>
+        <xdr:cNvPr id="2" name="AutoShape 2">
+          <a:extLst>
+            <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
+              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{ECEA1D74-1F4C-395C-E7A0-85FEBC60E597}"/>
+            </a:ext>
+          </a:extLst>
+        </xdr:cNvPr>
+        <xdr:cNvSpPr>
+          <a:spLocks noChangeArrowheads="1"/>
+        </xdr:cNvSpPr>
+      </xdr:nvSpPr>
+      <xdr:spPr bwMode="auto">
+        <a:xfrm>
+          <a:off x="0" y="0"/>
+          <a:ext cx="12700000" cy="12700000"/>
+        </a:xfrm>
+        <a:custGeom>
+          <a:avLst/>
+          <a:gdLst/>
+          <a:ahLst/>
+          <a:cxnLst/>
+          <a:rect l="0" t="0" r="0" b="0"/>
+          <a:pathLst/>
+        </a:custGeom>
+        <a:solidFill>
+          <a:srgbClr val="FFFFFF"/>
+        </a:solidFill>
+        <a:ln w="9525">
+          <a:solidFill>
+            <a:srgbClr val="000000"/>
+          </a:solidFill>
+          <a:round/>
+          <a:headEnd/>
+          <a:tailEnd/>
+        </a:ln>
+      </xdr:spPr>
+    </xdr:sp>
+    <xdr:clientData/>
+  </xdr:twoCellAnchor>
 </xdr:wsDr>
 </file>
 
@@ -2485,6 +3025,60 @@
             <a:srgbClr val="000000"/>
           </a:solidFill>
           <a:miter lim="800000"/>
+          <a:headEnd/>
+          <a:tailEnd/>
+        </a:ln>
+      </xdr:spPr>
+    </xdr:sp>
+    <xdr:clientData/>
+  </xdr:twoCellAnchor>
+  <xdr:twoCellAnchor>
+    <xdr:from>
+      <xdr:col>0</xdr:col>
+      <xdr:colOff>0</xdr:colOff>
+      <xdr:row>0</xdr:row>
+      <xdr:rowOff>0</xdr:rowOff>
+    </xdr:from>
+    <xdr:to>
+      <xdr:col>14</xdr:col>
+      <xdr:colOff>355600</xdr:colOff>
+      <xdr:row>66</xdr:row>
+      <xdr:rowOff>127000</xdr:rowOff>
+    </xdr:to>
+    <xdr:sp macro="" textlink="">
+      <xdr:nvSpPr>
+        <xdr:cNvPr id="2" name="AutoShape 2">
+          <a:extLst>
+            <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
+              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{F70219A0-8300-704C-4E5B-F8B6EF98CA0F}"/>
+            </a:ext>
+          </a:extLst>
+        </xdr:cNvPr>
+        <xdr:cNvSpPr>
+          <a:spLocks noChangeArrowheads="1"/>
+        </xdr:cNvSpPr>
+      </xdr:nvSpPr>
+      <xdr:spPr bwMode="auto">
+        <a:xfrm>
+          <a:off x="0" y="0"/>
+          <a:ext cx="12700000" cy="12700000"/>
+        </a:xfrm>
+        <a:custGeom>
+          <a:avLst/>
+          <a:gdLst/>
+          <a:ahLst/>
+          <a:cxnLst/>
+          <a:rect l="0" t="0" r="0" b="0"/>
+          <a:pathLst/>
+        </a:custGeom>
+        <a:solidFill>
+          <a:srgbClr val="FFFFFF"/>
+        </a:solidFill>
+        <a:ln w="9525">
+          <a:solidFill>
+            <a:srgbClr val="000000"/>
+          </a:solidFill>
+          <a:round/>
           <a:headEnd/>
           <a:tailEnd/>
         </a:ln>
@@ -2856,8 +3450,8 @@
       <c r="A5" s="1" t="s">
         <v>83</v>
       </c>
-      <c r="B5">
-        <v>1234</v>
+      <c r="B5" s="2">
+        <v>123</v>
       </c>
     </row>
   </sheetData>

</xml_diff>